<commit_message>
Fix height growth and establishment to match Fortran htgf.f and estab.f
- Remove artificial size/site dampening from potential height growth;
  Fortran uses raw Chapman-Richards with scale_factor=1.0 for SN
- Bound HTGMOD to [0.1, 2.0] (not individual HGMDRH to [0, 1])
  matching Fortran htgf.f combined modifier
- Remove extra competition modifier in tree.py _update_height_large_tree;
  Fortran HTGMOD (0.25*HGMDCR + 0.75*HGMDRH) is the sole modifier
- Remove BA floor (max 25.0) — pass actual BA to height growth model
- Add HHTMAX establishment height cap from estab.f/blkdat.f
- Fix TRAGE default from 1 to 2 (estab.f: IF(TRAGE.LT.0.5) TRAGE=2.0)
- Add non-SN variant scaling in establishment height calculation
- Fix NativeStand SITECODE column formatting and type hints
- Update compare_native.py to record initial state as cycle 1
- Regenerate test output files
</commit_message>
<xml_diff>
--- a/test_output/persistence_tests/yield_table.xlsx
+++ b/test_output/persistence_tests/yield_table.xlsx
@@ -508,37 +508,37 @@
         <v>500</v>
       </c>
       <c r="B2" t="n">
-        <v>0.03</v>
+        <v>18.12</v>
       </c>
       <c r="C2" t="n">
-        <v>0.09999999999999938</v>
+        <v>2.57765916184472</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1</v>
+        <v>2.56</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5</v>
+        <v>24.21679553771087</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5</v>
+        <v>20.18</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5000000000000003</v>
+        <v>1.438368595043547</v>
       </c>
       <c r="H2" t="n">
-        <v>0.308297500930738</v>
+        <v>56.75275090906761</v>
       </c>
       <c r="I2" t="n">
         <v>480</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>1.182348977272242</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L2" t="n">
-        <v>93.3</v>
+        <v>124.86</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -563,37 +563,37 @@
         <v>490</v>
       </c>
       <c r="B3" t="n">
-        <v>0.03</v>
+        <v>43.67</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1004999999999995</v>
+        <v>4.042239604403189</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1</v>
+        <v>4.03</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5</v>
+        <v>35.59809641123174</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5</v>
+        <v>30.64</v>
       </c>
       <c r="G3" t="n">
-        <v>0.002151230340764772</v>
+        <v>2.635377682066656</v>
       </c>
       <c r="H3" t="n">
-        <v>0.304559821414258</v>
+        <v>114.5050062524718</v>
       </c>
       <c r="I3" t="n">
         <v>480</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2.385520963593161</v>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>91.43000000000001</v>
+        <v>508.85</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -615,43 +615,43 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="B4" t="n">
-        <v>12.32</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>2.16060486385659</v>
+        <v>5.489384938887735</v>
       </c>
       <c r="D4" t="n">
-        <v>2.16</v>
+        <v>5.48</v>
       </c>
       <c r="E4" t="n">
-        <v>17.11057402324259</v>
+        <v>44.73999080579714</v>
       </c>
       <c r="F4" t="n">
-        <v>17.11</v>
+        <v>39.07</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9820978752441979</v>
+        <v>3.726867606950806</v>
       </c>
       <c r="H4" t="n">
-        <v>41.38460338782099</v>
+        <v>182.1603683220558</v>
       </c>
       <c r="I4" t="n">
         <v>480</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>3.795007673376162</v>
       </c>
       <c r="K4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L4" t="n">
-        <v>137.38</v>
+        <v>1195.33</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>637.3685556637834</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Fix SN hardwood growth gap: default ecounit 231T + Baskerville bias correction
Closes #5. Two root causes of 15-25% QMD underprediction vs native FVS:

1. Native FVS with state=0 defaults to S231T ecounit coefficients (habtyp.f:135).
   SN variant now defaults to ecounit '231T' when none specified, applying
   species-specific effects (LP: -0.183 slowdown, RO: +0.132 speedup).

2. Native FVS stochastic transform DDS*exp(Z) creates positive mean bias via
   Jensen's inequality. Added bounded Baskerville (1972) correction with α=0.88
   for ±2σ truncated normal, plus dgscor.f-style error suppression for large
   trees (no correction when ln(DDS) > 5.0, linear taper 4.0-5.0).

Results at 500 TPA SI=65 age 50 (QMD gap vs native):
- WO: -15% → -0.1%, RO: -20% → -10%, YP: -13% → -6%, SU: -20% → -10%
- LP now aligned at +2% (was over-predicting without S231T slowdown)
</commit_message>
<xml_diff>
--- a/test_output/persistence_tests/yield_table.xlsx
+++ b/test_output/persistence_tests/yield_table.xlsx
@@ -563,37 +563,37 @@
         <v>490</v>
       </c>
       <c r="B3" t="n">
-        <v>43.67</v>
+        <v>38.84</v>
       </c>
       <c r="C3" t="n">
-        <v>4.042239604403189</v>
+        <v>3.812262538983109</v>
       </c>
       <c r="D3" t="n">
-        <v>4.03</v>
+        <v>3.8</v>
       </c>
       <c r="E3" t="n">
-        <v>35.59809641123174</v>
+        <v>35.50937073315767</v>
       </c>
       <c r="F3" t="n">
-        <v>30.64</v>
+        <v>30.59</v>
       </c>
       <c r="G3" t="n">
-        <v>2.635377682066656</v>
+        <v>2.466042692939382</v>
       </c>
       <c r="H3" t="n">
-        <v>114.5050062524718</v>
+        <v>104.2304172952978</v>
       </c>
       <c r="I3" t="n">
         <v>480</v>
       </c>
       <c r="J3" t="n">
-        <v>2.385520963593161</v>
+        <v>2.171467026985372</v>
       </c>
       <c r="K3" t="n">
         <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>508.85</v>
+        <v>454.47</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -615,43 +615,43 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B4" t="n">
-        <v>78.40000000000001</v>
+        <v>66.45999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>5.489384938887735</v>
+        <v>5.043638641941123</v>
       </c>
       <c r="D4" t="n">
-        <v>5.48</v>
+        <v>5.03</v>
       </c>
       <c r="E4" t="n">
-        <v>44.73999080579714</v>
+        <v>44.59152314847052</v>
       </c>
       <c r="F4" t="n">
-        <v>39.07</v>
+        <v>39.02</v>
       </c>
       <c r="G4" t="n">
-        <v>3.726867606950806</v>
+        <v>3.360018405246064</v>
       </c>
       <c r="H4" t="n">
-        <v>182.1603683220558</v>
+        <v>159.6759742706182</v>
       </c>
       <c r="I4" t="n">
         <v>480</v>
       </c>
       <c r="J4" t="n">
-        <v>3.795007673376162</v>
+        <v>3.326582797304545</v>
       </c>
       <c r="K4" t="n">
         <v>15</v>
       </c>
       <c r="L4" t="n">
-        <v>1195.33</v>
+        <v>1014.54</v>
       </c>
       <c r="M4" t="n">
-        <v>637.3685556637834</v>
+        <v>293.7742581185481</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add PN/WC species-specific height-age curves from Fortran htcalc.f
PN/WC variants had no variant-specific small-tree height growth coefficients,
falling through to SN LP Chapman-Richards curves — causing 2-3x BA overshoot
vs native FVS. Implemented all 15 species-specific equation forms (King, Wiley,
Farr, Cochran, Hoyer, Alexander, Dolph, Herman, Barrett, Dahms, Curtis,
Harrington, Means, Cochran-424, Curtis misc) with WC overrides for DF/SS/RC.

WC DF Cycle 2 BA: 125.3 → 46.7 (native 47.4). PN DF BA MAPE: catastrophic → 27%.
222 regression tests pass, zero regressions on SN/LS/CS/NE.
</commit_message>
<xml_diff>
--- a/test_output/persistence_tests/yield_table.xlsx
+++ b/test_output/persistence_tests/yield_table.xlsx
@@ -508,37 +508,37 @@
         <v>500</v>
       </c>
       <c r="B2" t="n">
-        <v>18.12</v>
+        <v>16.4</v>
       </c>
       <c r="C2" t="n">
-        <v>2.57765916184472</v>
+        <v>2.451955101121936</v>
       </c>
       <c r="D2" t="n">
-        <v>2.56</v>
+        <v>2.45</v>
       </c>
       <c r="E2" t="n">
-        <v>24.21679553771087</v>
+        <v>20</v>
       </c>
       <c r="F2" t="n">
-        <v>20.18</v>
+        <v>19.3</v>
       </c>
       <c r="G2" t="n">
-        <v>1.438368595043547</v>
+        <v>1.306633359785076</v>
       </c>
       <c r="H2" t="n">
-        <v>56.75275090906761</v>
+        <v>52.37663440354625</v>
       </c>
       <c r="I2" t="n">
         <v>480</v>
       </c>
       <c r="J2" t="n">
-        <v>1.182348977272242</v>
+        <v>1.091179883407214</v>
       </c>
       <c r="K2" t="n">
         <v>5</v>
       </c>
       <c r="L2" t="n">
-        <v>124.86</v>
+        <v>103.58</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -560,40 +560,40 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B3" t="n">
-        <v>38.84</v>
+        <v>37.35</v>
       </c>
       <c r="C3" t="n">
-        <v>3.812262538983109</v>
+        <v>3.734490630182242</v>
       </c>
       <c r="D3" t="n">
-        <v>3.8</v>
+        <v>3.73</v>
       </c>
       <c r="E3" t="n">
-        <v>35.50937073315767</v>
+        <v>31.23415516255619</v>
       </c>
       <c r="F3" t="n">
-        <v>30.59</v>
+        <v>30.67</v>
       </c>
       <c r="G3" t="n">
-        <v>2.466042692939382</v>
+        <v>2.418129991116445</v>
       </c>
       <c r="H3" t="n">
-        <v>104.2304172952978</v>
+        <v>101.0445391797944</v>
       </c>
       <c r="I3" t="n">
         <v>480</v>
       </c>
       <c r="J3" t="n">
-        <v>2.171467026985372</v>
+        <v>2.105094566245716</v>
       </c>
       <c r="K3" t="n">
         <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>454.47</v>
+        <v>434.34</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -615,43 +615,43 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B4" t="n">
-        <v>66.45999999999999</v>
+        <v>65.08</v>
       </c>
       <c r="C4" t="n">
-        <v>5.043638641941123</v>
+        <v>5.001491830463586</v>
       </c>
       <c r="D4" t="n">
-        <v>5.03</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>44.59152314847052</v>
+        <v>40.38312685543093</v>
       </c>
       <c r="F4" t="n">
-        <v>39.02</v>
+        <v>39.77</v>
       </c>
       <c r="G4" t="n">
-        <v>3.360018405246064</v>
+        <v>3.31407455758902</v>
       </c>
       <c r="H4" t="n">
-        <v>159.6759742706182</v>
+        <v>156.8820222517913</v>
       </c>
       <c r="I4" t="n">
         <v>480</v>
       </c>
       <c r="J4" t="n">
-        <v>3.326582797304545</v>
+        <v>3.268375463578985</v>
       </c>
       <c r="K4" t="n">
         <v>15</v>
       </c>
       <c r="L4" t="n">
-        <v>1014.54</v>
+        <v>1005.66</v>
       </c>
       <c r="M4" t="n">
-        <v>293.7742581185481</v>
+        <v>244.6563624605441</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update test output and validation results after SN ecounit/establishment fix
Regenerated test outputs and native validation JSONs reflecting the
removal of ecounit from small-tree growth and SN establishment DBH
interpolation fix.
</commit_message>
<xml_diff>
--- a/test_output/persistence_tests/yield_table.xlsx
+++ b/test_output/persistence_tests/yield_table.xlsx
@@ -508,13 +508,13 @@
         <v>500</v>
       </c>
       <c r="B2" t="n">
-        <v>16.4</v>
+        <v>16.8</v>
       </c>
       <c r="C2" t="n">
-        <v>2.451955101121936</v>
+        <v>2.482360746042263</v>
       </c>
       <c r="D2" t="n">
-        <v>2.45</v>
+        <v>2.48</v>
       </c>
       <c r="E2" t="n">
         <v>20</v>
@@ -523,22 +523,22 @@
         <v>19.3</v>
       </c>
       <c r="G2" t="n">
-        <v>1.306633359785076</v>
+        <v>1.339240287458307</v>
       </c>
       <c r="H2" t="n">
-        <v>52.37663440354625</v>
+        <v>53.42298628199183</v>
       </c>
       <c r="I2" t="n">
         <v>480</v>
       </c>
       <c r="J2" t="n">
-        <v>1.091179883407214</v>
+        <v>1.11297888087483</v>
       </c>
       <c r="K2" t="n">
         <v>5</v>
       </c>
       <c r="L2" t="n">
-        <v>103.58</v>
+        <v>105.74</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -563,40 +563,40 @@
         <v>490</v>
       </c>
       <c r="B3" t="n">
-        <v>37.3</v>
+        <v>37.49</v>
       </c>
       <c r="C3" t="n">
-        <v>3.735818123011799</v>
+        <v>3.745330787684619</v>
       </c>
       <c r="D3" t="n">
         <v>3.73</v>
       </c>
       <c r="E3" t="n">
-        <v>31.23415516255619</v>
+        <v>31.29234814874847</v>
       </c>
       <c r="F3" t="n">
-        <v>30.68</v>
+        <v>30.61</v>
       </c>
       <c r="G3" t="n">
-        <v>2.414172568243151</v>
+        <v>2.415237973035909</v>
       </c>
       <c r="H3" t="n">
-        <v>100.8962831870018</v>
+        <v>101.3089513364138</v>
       </c>
       <c r="I3" t="n">
         <v>480</v>
       </c>
       <c r="J3" t="n">
-        <v>2.102005899729203</v>
+        <v>2.110603152841954</v>
       </c>
       <c r="K3" t="n">
         <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>433.89</v>
+        <v>435.62</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>0.6040686510442865</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -615,43 +615,43 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="B4" t="n">
-        <v>65.16</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>5.00463451698771</v>
+        <v>4.964577029598355</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>4.93</v>
       </c>
       <c r="E4" t="n">
-        <v>40.38312685543093</v>
+        <v>40.1967600774659</v>
       </c>
       <c r="F4" t="n">
-        <v>39.79</v>
+        <v>39.68</v>
       </c>
       <c r="G4" t="n">
-        <v>3.316704768892213</v>
+        <v>3.307103083224905</v>
       </c>
       <c r="H4" t="n">
-        <v>157.0402680726012</v>
+        <v>156.6527615198173</v>
       </c>
       <c r="I4" t="n">
         <v>480</v>
       </c>
       <c r="J4" t="n">
-        <v>3.271672251512525</v>
+        <v>3.263599198329528</v>
       </c>
       <c r="K4" t="n">
         <v>15</v>
       </c>
       <c r="L4" t="n">
-        <v>1007.27</v>
+        <v>1000.69</v>
       </c>
       <c r="M4" t="n">
-        <v>247.2606867627731</v>
+        <v>288.4988598054628</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Fix PN/WC height growth to use forward increment matching Fortran htgf.f
The POTHTG calculation for PN/WC variants was using a backward 5-year
height increment H(age) - H(age-5) instead of the correct forward
increment H(age+5) - H(age). On concave-down height-age curves, the
backward increment systematically overestimates height growth, causing
cumulative top height overprediction.

Results (single-run, deterministic comparison vs native FVS):
- PN DF top_height MAE: 3.30' -> 1.15' (-65%)
- WC DF top_height MAE: 1.07' -> 0.52' (-51%)
- PN DF volume MAPE: 10.6% -> 5.9% (now passes 10% threshold)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_output/persistence_tests/yield_table.xlsx
+++ b/test_output/persistence_tests/yield_table.xlsx
@@ -563,40 +563,40 @@
         <v>490</v>
       </c>
       <c r="B3" t="n">
-        <v>37.49</v>
+        <v>38.16</v>
       </c>
       <c r="C3" t="n">
-        <v>3.745330787684619</v>
+        <v>3.778542235526446</v>
       </c>
       <c r="D3" t="n">
-        <v>3.73</v>
+        <v>3.76</v>
       </c>
       <c r="E3" t="n">
-        <v>31.29234814874847</v>
+        <v>31.32621045873878</v>
       </c>
       <c r="F3" t="n">
-        <v>30.61</v>
+        <v>30.63</v>
       </c>
       <c r="G3" t="n">
-        <v>2.415237973035909</v>
+        <v>2.43837243869552</v>
       </c>
       <c r="H3" t="n">
-        <v>101.3089513364138</v>
+        <v>102.7546657906387</v>
       </c>
       <c r="I3" t="n">
         <v>480</v>
       </c>
       <c r="J3" t="n">
-        <v>2.110603152841954</v>
+        <v>2.14072220397164</v>
       </c>
       <c r="K3" t="n">
         <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>435.62</v>
+        <v>443.23</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6040686510442865</v>
+        <v>1.277882837114802</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -618,40 +618,40 @@
         <v>482</v>
       </c>
       <c r="B4" t="n">
-        <v>64.79000000000001</v>
+        <v>65.48</v>
       </c>
       <c r="C4" t="n">
-        <v>4.964577029598355</v>
+        <v>4.990857120706463</v>
       </c>
       <c r="D4" t="n">
-        <v>4.93</v>
+        <v>4.95</v>
       </c>
       <c r="E4" t="n">
-        <v>40.1967600774659</v>
+        <v>40.25164264959943</v>
       </c>
       <c r="F4" t="n">
-        <v>39.68</v>
+        <v>39.69</v>
       </c>
       <c r="G4" t="n">
-        <v>3.307103083224905</v>
+        <v>3.327162464146378</v>
       </c>
       <c r="H4" t="n">
-        <v>156.6527615198173</v>
+        <v>157.9858288863996</v>
       </c>
       <c r="I4" t="n">
         <v>480</v>
       </c>
       <c r="J4" t="n">
-        <v>3.263599198329528</v>
+        <v>3.291371435133324</v>
       </c>
       <c r="K4" t="n">
         <v>15</v>
       </c>
       <c r="L4" t="n">
-        <v>1000.69</v>
+        <v>1011.06</v>
       </c>
       <c r="M4" t="n">
-        <v>288.4988598054628</v>
+        <v>313.2099462108267</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>

</xml_diff>